<commit_message>
Otomatik veri güncelleme (18.09.2026 15:11 UTC)
</commit_message>
<xml_diff>
--- a/net rezerv/net_rezerv.xlsx
+++ b/net rezerv/net_rezerv.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1183"/>
+  <dimension ref="A1:R1184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -66704,6 +66704,62 @@
         <v>4865747024</v>
       </c>
     </row>
+    <row r="1184">
+      <c r="A1184" s="1" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B1184" t="n">
+        <v>48.5779</v>
+      </c>
+      <c r="C1184" t="n">
+        <v>176112.7682958712</v>
+      </c>
+      <c r="D1184" t="n">
+        <v>83361.44965097298</v>
+      </c>
+      <c r="E1184" t="n">
+        <v>259474.2179468442</v>
+      </c>
+      <c r="F1184" t="n">
+        <v>58965.94924852659</v>
+      </c>
+      <c r="G1184" t="n">
+        <v>14894.83024173544</v>
+      </c>
+      <c r="H1184" t="n">
+        <v>5481.908789799477</v>
+      </c>
+      <c r="I1184" t="n">
+        <v>102309.7508331978</v>
+      </c>
+      <c r="J1184" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1184" t="n">
+        <v>3754.76</v>
+      </c>
+      <c r="L1184" t="n">
+        <v>-3754.76</v>
+      </c>
+      <c r="M1184" t="n">
+        <v>53426.27843113843</v>
+      </c>
+      <c r="N1184" t="n">
+        <v>57181.03843113843</v>
+      </c>
+      <c r="O1184" t="n">
+        <v>8555188447</v>
+      </c>
+      <c r="P1184" t="n">
+        <v>723559574</v>
+      </c>
+      <c r="Q1184" t="n">
+        <v>266299617</v>
+      </c>
+      <c r="R1184" t="n">
+        <v>4969992845</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Otomatik veri güncelleme (09.10.2026 17:35 UTC)
</commit_message>
<xml_diff>
--- a/net rezerv/net_rezerv.xlsx
+++ b/net rezerv/net_rezerv.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1198"/>
+  <dimension ref="A1:R1199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -67535,6 +67535,62 @@
       </c>
       <c r="R1198" t="n">
         <v>4865444955</v>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" s="1" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B1199" t="n">
+        <v>49.1091</v>
+      </c>
+      <c r="C1199" t="n">
+        <v>174724.1725260695</v>
+      </c>
+      <c r="D1199" t="n">
+        <v>107062.0168102</v>
+      </c>
+      <c r="E1199" t="n">
+        <v>174724.1725260695</v>
+      </c>
+      <c r="F1199" t="n">
+        <v>51582.83147115301</v>
+      </c>
+      <c r="G1199" t="n">
+        <v>17496.35955454285</v>
+      </c>
+      <c r="H1199" t="n">
+        <v>7177.744918966138</v>
+      </c>
+      <c r="I1199" t="n">
+        <v>98467.23658140752</v>
+      </c>
+      <c r="J1199" t="n">
+        <v>0</v>
+      </c>
+      <c r="K1199" t="n">
+        <v>2876.40475</v>
+      </c>
+      <c r="L1199" t="n">
+        <v>-2876.40475</v>
+      </c>
+      <c r="M1199" t="n">
+        <v>51582.83147115301</v>
+      </c>
+      <c r="N1199" t="n">
+        <v>54459.23622115301</v>
+      </c>
+      <c r="O1199" t="n">
+        <v>8580546861</v>
+      </c>
+      <c r="P1199" t="n">
+        <v>859230471</v>
+      </c>
+      <c r="Q1199" t="n">
+        <v>352492593</v>
+      </c>
+      <c r="R1199" t="n">
+        <v>4835637368</v>
       </c>
     </row>
   </sheetData>

</xml_diff>